<commit_message>
Regenerate with green palette
</commit_message>
<xml_diff>
--- a/buyict_email_registry.xlsx
+++ b/buyict_email_registry.xlsx
@@ -29,10 +29,7 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00B8860B"/>
-    </font>
+    <font/>
   </fonts>
   <fills count="4">
     <fill>
@@ -43,12 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001C1C1C"/>
+        <fgColor rgb="0019473C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFACD"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,16 +59,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0E0DC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0E0DC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0E0DC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0E0DC"/>
       </bottom>
     </border>
   </borders>

</xml_diff>